<commit_message>
Major update, private data now fully supported.
</commit_message>
<xml_diff>
--- a/data/primers/Demo Primers.xlsx
+++ b/data/primers/Demo Primers.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\loa012\Python\PYEAST\data\primers\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\u5390772\Desktop\Code\PYEAST Local\data\primers\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{463DE22D-6C0C-405F-98CE-97A98325CEAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F76317F4-13C9-4EF1-BAAE-66AB53913D2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11620" xr2:uid="{3674F192-AC5C-47E2-8A02-E860BFF3F7B0}"/>
+    <workbookView xWindow="-27765" yWindow="2670" windowWidth="16410" windowHeight="11295" xr2:uid="{3674F192-AC5C-47E2-8A02-E860BFF3F7B0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -650,7 +650,7 @@
     <t>His3MX_down_R</t>
   </si>
   <si>
-    <t>cctcgttcagaatgacacgtata</t>
+    <t>cctcgttcagaatgacacg</t>
   </si>
 </sst>
 </file>
@@ -1061,15 +1061,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02F98113-4DF1-41D8-8ACA-74C6010B1D34}">
   <dimension ref="A1:D97"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.08984375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.36328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.08984375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.81640625" customWidth="1"/>
+    <col min="1" max="1" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="14" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1083,7 +1083,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -1097,7 +1097,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -1111,7 +1111,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -1125,7 +1125,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -1139,7 +1139,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -1153,7 +1153,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>4</v>
       </c>
@@ -1167,7 +1167,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>4</v>
       </c>
@@ -1181,7 +1181,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>4</v>
       </c>
@@ -1195,7 +1195,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>4</v>
       </c>
@@ -1209,7 +1209,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>4</v>
       </c>
@@ -1223,7 +1223,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>4</v>
       </c>
@@ -1237,7 +1237,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>4</v>
       </c>
@@ -1251,7 +1251,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>4</v>
       </c>
@@ -1265,7 +1265,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>4</v>
       </c>
@@ -1279,7 +1279,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>4</v>
       </c>
@@ -1293,7 +1293,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>4</v>
       </c>
@@ -1307,7 +1307,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>4</v>
       </c>
@@ -1321,7 +1321,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>4</v>
       </c>
@@ -1335,7 +1335,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>4</v>
       </c>
@@ -1349,7 +1349,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>4</v>
       </c>
@@ -1363,7 +1363,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>4</v>
       </c>
@@ -1377,7 +1377,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>4</v>
       </c>
@@ -1391,7 +1391,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>4</v>
       </c>
@@ -1405,7 +1405,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>4</v>
       </c>
@@ -1419,7 +1419,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>4</v>
       </c>
@@ -1433,7 +1433,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>4</v>
       </c>
@@ -1447,7 +1447,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>4</v>
       </c>
@@ -1461,7 +1461,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>4</v>
       </c>
@@ -1475,7 +1475,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>4</v>
       </c>
@@ -1489,7 +1489,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>4</v>
       </c>
@@ -1503,7 +1503,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>4</v>
       </c>
@@ -1517,7 +1517,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>4</v>
       </c>
@@ -1531,7 +1531,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>4</v>
       </c>
@@ -1545,7 +1545,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>4</v>
       </c>
@@ -1559,7 +1559,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>4</v>
       </c>
@@ -1573,7 +1573,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>4</v>
       </c>
@@ -1587,7 +1587,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>4</v>
       </c>
@@ -1601,7 +1601,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>4</v>
       </c>
@@ -1615,7 +1615,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>4</v>
       </c>
@@ -1629,7 +1629,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>4</v>
       </c>
@@ -1643,7 +1643,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>4</v>
       </c>
@@ -1657,7 +1657,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>4</v>
       </c>
@@ -1671,7 +1671,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>4</v>
       </c>
@@ -1685,7 +1685,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>4</v>
       </c>
@@ -1699,7 +1699,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>4</v>
       </c>
@@ -1713,7 +1713,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>4</v>
       </c>
@@ -1727,7 +1727,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>4</v>
       </c>
@@ -1741,7 +1741,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>4</v>
       </c>
@@ -1755,7 +1755,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>4</v>
       </c>
@@ -1769,7 +1769,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>4</v>
       </c>
@@ -1783,7 +1783,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>4</v>
       </c>
@@ -1797,7 +1797,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>4</v>
       </c>
@@ -1811,7 +1811,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>4</v>
       </c>
@@ -1819,7 +1819,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>4</v>
       </c>
@@ -1827,7 +1827,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>4</v>
       </c>
@@ -1835,7 +1835,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>4</v>
       </c>
@@ -1843,7 +1843,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>4</v>
       </c>
@@ -1851,7 +1851,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>4</v>
       </c>
@@ -1859,7 +1859,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>4</v>
       </c>
@@ -1867,7 +1867,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>4</v>
       </c>
@@ -1875,7 +1875,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>4</v>
       </c>
@@ -1883,7 +1883,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>4</v>
       </c>
@@ -1891,7 +1891,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>4</v>
       </c>
@@ -1899,7 +1899,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>4</v>
       </c>
@@ -1907,7 +1907,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>4</v>
       </c>
@@ -1915,7 +1915,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>4</v>
       </c>
@@ -1923,7 +1923,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>4</v>
       </c>
@@ -1931,7 +1931,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>4</v>
       </c>
@@ -1939,7 +1939,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>4</v>
       </c>
@@ -1947,7 +1947,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>4</v>
       </c>
@@ -1955,7 +1955,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>4</v>
       </c>
@@ -1963,7 +1963,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>4</v>
       </c>
@@ -1971,7 +1971,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>4</v>
       </c>
@@ -1979,7 +1979,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>4</v>
       </c>
@@ -1987,7 +1987,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>4</v>
       </c>
@@ -1995,7 +1995,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>4</v>
       </c>
@@ -2003,7 +2003,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>4</v>
       </c>
@@ -2011,7 +2011,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>4</v>
       </c>
@@ -2019,7 +2019,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>4</v>
       </c>
@@ -2027,7 +2027,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="81" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>4</v>
       </c>
@@ -2035,7 +2035,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="82" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>4</v>
       </c>
@@ -2043,7 +2043,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="83" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>4</v>
       </c>
@@ -2051,7 +2051,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="84" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>4</v>
       </c>
@@ -2059,7 +2059,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="85" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>4</v>
       </c>
@@ -2067,7 +2067,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="86" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>4</v>
       </c>
@@ -2075,7 +2075,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="87" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>4</v>
       </c>
@@ -2083,7 +2083,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="88" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>4</v>
       </c>
@@ -2091,7 +2091,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="89" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>4</v>
       </c>
@@ -2099,7 +2099,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="90" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>4</v>
       </c>
@@ -2107,7 +2107,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="91" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>4</v>
       </c>
@@ -2115,7 +2115,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="92" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>4</v>
       </c>
@@ -2123,7 +2123,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="93" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>4</v>
       </c>
@@ -2131,7 +2131,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="94" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>4</v>
       </c>
@@ -2139,7 +2139,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="95" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>4</v>
       </c>
@@ -2147,7 +2147,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="96" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>4</v>
       </c>
@@ -2155,7 +2155,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="97" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>4</v>
       </c>

</xml_diff>